<commit_message>
Demo: a whole fake term through every adapter that can parse offline
hub/demo.py now replays one fake student's full UBC term (13 teaching
weeks + a 2-week exam period, `now` always in week 5) through the real
Canvas, calendar-feed, PrairieLearn, WeBWorK, Brightspace, Piazza,
Workday (courses + schedule), Bookstore and key-dates parsers. Fixtures
are in each provider's own response shape with date tokens rendered at
request time ({{due:+1d@23:59}}, {{due:w6.Tue@18:00}}, {{date:w1.Tue}}).

demo_rows() also returns "schedule" (/api/schedule's shape) and
"textbooks". Tests cover the term span, every kind, cross-source dedupe,
course-code matching, overdue/urgency, same-day clusters, the 23:59
Vancouver edge, weekday stability and determinism.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KLtrzHK6UkLsBgfMydXv5j
</commit_message>
<xml_diff>
--- a/hub/demo_fixtures/workday_view_my_courses.xlsx
+++ b/hub/demo_fixtures/workday_view_my_courses.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -505,7 +505,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Demo Student (00000000) - Faculty of Demo Studies/Undergraduate - 2026-01-01 - Active - CPSC 110 - Intro to Program Design (Demo)</t>
+          <t>Stu Dent (00000000) - Faculty of Demo Studies/Undergraduate - 2026-01-01 - Active - CPSC 110 - Intro to Program Design (Demo)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-09-08 - 2026-12-05 | Mon Wed Fri | 10:00 a.m. - 11:00 a.m. | Demo Building (DEMO) | Floor: 1 | Room: 100</t>
+          <t>{{date:w1.Tue}} - {{date:w13.Fri}} | Mon Wed Fri | 10:00 a.m. - 11:00 a.m. | Demo Hall (DEMO) | Floor: 1 | Room: 110</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -553,19 +553,19 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>{{date:w1.Tue}}</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-12-05</t>
+          <t>{{date:w13.Fri}}</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Demo Student (00000000) - Faculty of Demo Studies/Undergraduate - 2026-01-01 - Active - CPSC 110 - Intro to Program Design (Demo)</t>
+          <t>Stu Dent (00000000) - Faculty of Demo Studies/Undergraduate - 2026-01-01 - Active - CPSC 110 - Intro to Program Design (Demo)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -603,34 +603,34 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-09-08 - 2026-12-05 | Tue | 2:00 p.m. - 4:00 p.m. | Demo Building (DEMO) | Floor: 1 | Room: 100</t>
+          <t>{{date:w1.Tue}} - {{date:w13.Fri}} | Mon | 2:00 p.m. - 4:00 p.m. | Demo Computing Lab (DCL) | Floor: B | Room: 005</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>D. Instructor</t>
+          <t>T. Assistant</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>{{date:w1.Tue}}</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-12-05</t>
+          <t>{{date:w13.Fri}}</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Demo Student (00000000) - Faculty of Demo Studies/Undergraduate - 2026-01-01 - Active - MATH 101 - Integral Calculus (Demo)</t>
+          <t>Stu Dent (00000000) - Faculty of Demo Studies/Undergraduate - 2026-01-01 - Active - CPSC 110 - Intro to Program Design (Demo)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MATH 101 - Integral Calculus (Demo)</t>
+          <t>CPSC 110 - Intro to Program Design (Demo)</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -643,7 +643,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>MATH 101-102 - Integral Calculus (Demo)</t>
+          <t>CPSC 110-101 - Intro to Program Design (Demo)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Lecture</t>
+          <t>Final Exam</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -663,34 +663,34 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-09-08 - 2026-12-05 | Tue Thu | 9:30 a.m. - 11:00 a.m. | Demo Building (DEMO) | Floor: 1 | Room: 100</t>
+          <t>{{date:w14.Wed}} - {{date:w14.Wed}} | Wed | 12:00 p.m. - 2:30 p.m. | Demo Hall (DEMO) | Floor: 1 | Room: 200</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>E. Lecturer</t>
+          <t>D. Instructor</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>{{date:w1.Tue}}</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-12-05</t>
+          <t>{{date:w13.Fri}}</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Demo Student (00000000) - Faculty of Demo Studies/Undergraduate - 2026-01-01 - Active - ENGL 110 - Approaches to Stories (Demo)</t>
+          <t>Stu Dent (00000000) - Faculty of Demo Studies/Undergraduate - 2026-01-01 - Active - MATH 100 - Differential Calculus (Demo)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ENGL 110 - Approaches to Stories (Demo)</t>
+          <t>MATH 100 - Differential Calculus (Demo)</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -703,7 +703,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>ENGL 110-001 - Approaches to Stories (Demo)</t>
+          <t>MATH 100-104 - Differential Calculus (Demo)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -723,34 +723,34 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-09-08 - 2026-12-05 | Mon Wed | 1:00 p.m. - 2:30 p.m. | Demo Building (DEMO) | Floor: 1 | Room: 100</t>
+          <t>{{date:w1.Tue}} - {{date:w13.Fri}} | Tue Thu | 9:30 a.m. - 11:00 a.m. | Demo Math Annex (DMA) | Floor: 1 | Room: 100</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>F. Professor</t>
+          <t>E. Lecturer</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>{{date:w1.Tue}}</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-12-05</t>
+          <t>{{date:w13.Fri}}</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Demo Student (00000000) - Faculty of Demo Studies/Undergraduate - 2026-01-01 - Active - PSYC 102 - Intro to Minds (Demo)</t>
+          <t>Stu Dent (00000000) - Faculty of Demo Studies/Undergraduate - 2026-01-01 - Active - MATH 100 - Differential Calculus (Demo)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PSYC 102 - Intro to Minds (Demo)</t>
+          <t>MATH 100 - Differential Calculus (Demo)</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -763,42 +763,282 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
+          <t>MATH 100-T4C - Differential Calculus (Demo)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Discussion</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>In Person Learning</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>{{date:w1.Tue}} - {{date:w13.Fri}} | Fri | 1:00 p.m. - 2:00 p.m. | Demo Math Annex (DMA) | Floor: 2 | Room: 204</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>T. Assistant</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>{{date:w1.Tue}}</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>{{date:w13.Fri}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Stu Dent (00000000) - Faculty of Demo Studies/Undergraduate - 2026-01-01 - Active - PHYS 117 - Dynamics and Waves (Demo)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PHYS 117 - Dynamics and Waves (Demo)</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Graded</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>PHYS 117-101 - Dynamics and Waves (Demo)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>In Person Learning</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>{{date:w1.Tue}} - {{date:w13.Fri}} | Mon Wed Fri | 12:00 p.m. - 1:00 p.m. | Demo Physics Hall (DPH) | Floor: 1 | Room: 101</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>F. Professor</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>{{date:w1.Tue}}</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>{{date:w13.Fri}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Stu Dent (00000000) - Faculty of Demo Studies/Undergraduate - 2026-01-01 - Active - PHYS 117 - Dynamics and Waves (Demo)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PHYS 117 - Dynamics and Waves (Demo)</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Graded</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>PHYS 117-L2B - Dynamics and Waves (Demo)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>In Person Learning</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>{{date:w1.Tue}} - {{date:w13.Fri}} | Thu | 3:00 p.m. - 6:00 p.m. | Demo Physics Hall (DPH) | Floor: 3 | Room: 310</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>T. Assistant</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>{{date:w1.Tue}}</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>{{date:w13.Fri}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Stu Dent (00000000) - Faculty of Demo Studies/Undergraduate - 2026-01-01 - Active - ENGL 110 - Approaches to Stories (Demo)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ENGL 110 - Approaches to Stories (Demo)</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Graded</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>ENGL 110-003 - Approaches to Stories (Demo)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Seminar</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>In Person Learning</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>{{date:w1.Tue}} - {{date:w13.Fri}} | Tue Thu | 12:30 p.m. - 2:00 p.m. | Demo Arts Building (DAB) | Floor: 2 | Room: 200</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>G. Teacher</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>{{date:w1.Tue}}</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>{{date:w13.Fri}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Stu Dent (00000000) - Faculty of Demo Studies/Undergraduate - 2026-01-01 - Active - PSYC 102 - Intro to Minds (Demo)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PSYC 102 - Intro to Minds (Demo)</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Graded</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>PSYC 102-003 - Intro to Minds (Demo)</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Registered</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Lecture</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>In Person Learning</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>2026-09-08 - 2026-12-05 | Tue Thu | 3:30 p.m. - 5:00 p.m. | Demo Building (DEMO) | Floor: 1 | Room: 100</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>G. Teacher</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>2026-12-05</t>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>{{date:w1.Tue}} - {{date:w13.Fri}} | Tue Thu | 3:30 p.m. - 5:00 p.m. | Demo Lecture Theatre (DLT) | Floor: 1 | Room: 1</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>H. Researcher</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>{{date:w1.Tue}}</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>{{date:w13.Fri}}</t>
         </is>
       </c>
     </row>

</xml_diff>